<commit_message>
subindo a modelagem e iniciando a tela de quiz
</commit_message>
<xml_diff>
--- a/documentação/backlog.xlsx
+++ b/documentação/backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\josue\Documents\Josué Alvarez\Jach-a-Ajayu\documentação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{396F0273-5582-4600-803D-80FDA668FB6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6582A087-172E-4637-B715-A56954B51519}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="64">
   <si>
     <t>Requisito</t>
   </si>
@@ -222,6 +222,12 @@
   </si>
   <si>
     <t>Criar o site de quis com as perguntas sobre as danças da Bolivia</t>
+  </si>
+  <si>
+    <t>Site Minha História</t>
+  </si>
+  <si>
+    <t>Criar o site contando minha história na dança</t>
   </si>
 </sst>
 </file>
@@ -677,7 +683,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="4"/>
@@ -780,15 +786,15 @@
         <v>55</v>
       </c>
       <c r="L3" s="7">
-        <f>SUM(F3:F19)</f>
-        <v>169</v>
+        <f>SUM(F3:F20)</f>
+        <v>177</v>
       </c>
       <c r="M3" s="7">
         <v>0</v>
       </c>
       <c r="N3" s="7">
         <f>L3</f>
-        <v>169</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -824,15 +830,15 @@
       </c>
       <c r="L4" s="7">
         <f>L3-M3</f>
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="M4" s="7">
-        <f>SUMIFS(F3:F19,I3:I19,TRUE,H3:H19,"27/10 - 31/10")</f>
+        <f>SUMIFS(F3:F20,I3:I20,TRUE,H3:H20,"27/10 - 31/10")</f>
         <v>19</v>
       </c>
       <c r="N4" s="7">
         <f>L4-M4</f>
-        <v>150</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -868,15 +874,15 @@
       </c>
       <c r="L5" s="7">
         <f t="shared" ref="L5:L8" si="0">L4-M4</f>
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="M5" s="7">
-        <f>SUMIFS(F3:F19,I3:I19,TRUE,H3:H19,"03/11 - 07/11")</f>
+        <f>SUMIFS(F3:F20,I3:I20,TRUE,H3:H20,"03/11 - 07/11")</f>
         <v>16</v>
       </c>
       <c r="N5" s="7">
-        <f t="shared" ref="N5:N7" si="1">L5-M5</f>
-        <v>134</v>
+        <f t="shared" ref="N5" si="1">L5-M5</f>
+        <v>142</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -912,15 +918,15 @@
       </c>
       <c r="L6" s="7">
         <f t="shared" si="0"/>
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="M6" s="7">
-        <f>SUMIFS(F3:F19,I3:I19,TRUE,H3:H19,"10/11 - 14/11")</f>
+        <f>SUMIFS(F3:F20,I3:I20,TRUE,H3:H20,"10/11 - 14/11")</f>
         <v>29</v>
       </c>
       <c r="N6" s="7">
         <f>L6-M6</f>
-        <v>105</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -956,11 +962,11 @@
       </c>
       <c r="L7" s="7">
         <f t="shared" si="0"/>
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="M7" s="7">
-        <f>SUMIFS(F3:F19,I3:I19,TRUE,H3:H19,"17/11 - 21/11")</f>
-        <v>0</v>
+        <f>SUMIFS(F3:F20,I3:I20,TRUE,H3:H20,"17/11 - 21/11")</f>
+        <v>8</v>
       </c>
       <c r="N7" s="7">
         <f>L7-M7</f>
@@ -1088,9 +1094,11 @@
       <c r="G11" s="4">
         <v>2</v>
       </c>
-      <c r="H11" s="7"/>
+      <c r="H11" s="7" t="s">
+        <v>54</v>
+      </c>
       <c r="I11" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K11" s="7"/>
     </row>
@@ -1170,7 +1178,7 @@
         <v>8</v>
       </c>
       <c r="G14" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H14" s="7" t="s">
         <v>53</v>
@@ -1184,10 +1192,10 @@
         <v>13</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>15</v>
+        <v>62</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>22</v>
@@ -1199,13 +1207,11 @@
         <v>8</v>
       </c>
       <c r="G15" s="4">
-        <v>1</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>53</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="H15" s="7"/>
       <c r="I15" s="5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -1213,22 +1219,22 @@
         <v>14</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>22</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F16" s="4">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="G16" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H16" s="7" t="s">
         <v>53</v>
@@ -1242,37 +1248,39 @@
         <v>15</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>22</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F17" s="4">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="G17" s="4">
-        <v>1</v>
-      </c>
-      <c r="H17" s="7"/>
+        <v>2</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>53</v>
+      </c>
       <c r="I17" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <v>16</v>
       </c>
-      <c r="B18" s="6" t="s">
-        <v>60</v>
+      <c r="B18" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>22</v>
@@ -1295,26 +1303,53 @@
       <c r="A19" s="4">
         <v>17</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>28</v>
+      <c r="B19" s="6" t="s">
+        <v>60</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>22</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F19" s="4">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="G19" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H19" s="7"/>
       <c r="I19" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="4">
+        <v>18</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F20" s="4">
+        <v>13</v>
+      </c>
+      <c r="G20" s="4">
+        <v>2</v>
+      </c>
+      <c r="H20" s="7"/>
+      <c r="I20" s="5" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Interligando a API com o Quiz e a Dashboard
</commit_message>
<xml_diff>
--- a/documentação/backlog.xlsx
+++ b/documentação/backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\josue\Documents\Josué Alvarez\Jach-a-Ajayu\documentação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6582A087-172E-4637-B715-A56954B51519}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9C4BCF7-096B-4744-9124-FC60064A2AB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="65">
   <si>
     <t>Requisito</t>
   </si>
@@ -218,9 +218,6 @@
     <t>JACH'A AJAYU</t>
   </si>
   <si>
-    <t>Site Quiz Conhecimento das Danças</t>
-  </si>
-  <si>
     <t>Criar o site de quis com as perguntas sobre as danças da Bolivia</t>
   </si>
   <si>
@@ -228,12 +225,21 @@
   </si>
   <si>
     <t>Criar o site contando minha história na dança</t>
+  </si>
+  <si>
+    <t>% de Conclusão</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site Quiz </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="169" formatCode="0.0"/>
+  </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -295,7 +301,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -324,6 +330,9 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -696,7 +705,7 @@
     <col min="8" max="8" width="12.140625" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="9.140625" style="3"/>
     <col min="11" max="11" width="12.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="11" style="3" bestFit="1" customWidth="1"/>
     <col min="15" max="16384" width="9.140625" style="3"/>
@@ -966,11 +975,11 @@
       </c>
       <c r="M7" s="7">
         <f>SUMIFS(F3:F20,I3:I20,TRUE,H3:H20,"17/11 - 21/11")</f>
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="N7" s="7">
         <f>L7-M7</f>
-        <v>105</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -1006,7 +1015,7 @@
       </c>
       <c r="L8" s="7">
         <f t="shared" si="0"/>
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="M8" s="7" t="s">
         <v>23</v>
@@ -1066,11 +1075,19 @@
       <c r="G10" s="4">
         <v>3</v>
       </c>
-      <c r="H10" s="7"/>
+      <c r="H10" s="7" t="s">
+        <v>54</v>
+      </c>
       <c r="I10" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="K10" s="7"/>
+        <v>1</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="L10" s="11">
+        <f>13/18*100</f>
+        <v>72.222222222222214</v>
+      </c>
     </row>
     <row r="11" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
@@ -1192,10 +1209,10 @@
         <v>13</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>62</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>63</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>22</v>
@@ -1209,9 +1226,11 @@
       <c r="G15" s="4">
         <v>2</v>
       </c>
-      <c r="H15" s="7"/>
+      <c r="H15" s="7" t="s">
+        <v>54</v>
+      </c>
       <c r="I15" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -1304,10 +1323,10 @@
         <v>17</v>
       </c>
       <c r="B19" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C19" s="6" t="s">
         <v>60</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>61</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>22</v>
@@ -1323,7 +1342,7 @@
       </c>
       <c r="H19" s="7"/>
       <c r="I19" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
FInalizando Documentação e Backlog
</commit_message>
<xml_diff>
--- a/documentação/backlog.xlsx
+++ b/documentação/backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\josue\Documents\Josué Alvarez\Jach-a-Ajayu\documentação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A1C72D8-ECD8-4B95-B160-E47A44849412}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84B8FEC7-142F-462C-8FE8-C6D6B25844EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="65">
   <si>
     <t>Requisito</t>
   </si>
@@ -500,10 +500,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -966,9 +966,11 @@
       <c r="H4" s="11">
         <v>2</v>
       </c>
-      <c r="I4" s="11"/>
+      <c r="I4" s="11" t="s">
+        <v>54</v>
+      </c>
       <c r="J4" s="12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L4" s="13" t="s">
         <v>55</v>
@@ -1154,11 +1156,11 @@
       </c>
       <c r="N8" s="11">
         <f>SUMIFS(G4:G21,J4:J21,TRUE,I4:I21,"17/11 - 21/11")</f>
-        <v>97</v>
+        <v>113</v>
       </c>
       <c r="O8" s="14">
         <f>M8-N8</f>
-        <v>16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="2:15" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -1194,7 +1196,7 @@
       </c>
       <c r="M9" s="16">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="N9" s="16" t="s">
         <v>23</v>
@@ -1260,13 +1262,13 @@
       <c r="J11" s="12" t="b">
         <v>1</v>
       </c>
-      <c r="L11" s="23" t="s">
+      <c r="L11" s="24" t="s">
         <v>63</v>
       </c>
-      <c r="M11" s="23"/>
-      <c r="N11" s="24">
+      <c r="M11" s="24"/>
+      <c r="N11" s="23">
         <f>COUNTIF(J4:J21,TRUE)/18</f>
-        <v>0.88888888888888884</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="2:15" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -1321,9 +1323,11 @@
       <c r="H13" s="11">
         <v>2</v>
       </c>
-      <c r="I13" s="11"/>
+      <c r="I13" s="11" t="s">
+        <v>54</v>
+      </c>
       <c r="J13" s="12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L13" s="3"/>
     </row>

</xml_diff>